<commit_message>
fixed bugs with sensitivity. Long version prior to clean up
</commit_message>
<xml_diff>
--- a/Distributions/Sensitivity.xlsx
+++ b/Distributions/Sensitivity.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://esait-my.sharepoint.com/personal/ivo_ferreira_esa_int/Documents/NewAthenaE2EPSF_v3/Distributions/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="32" documentId="14_{6BA1779D-2885-C748-8AC6-FE991EB9936B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9BD2354D-6FCB-AF4A-A251-116AA03F05E7}"/>
+  <xr:revisionPtr revIDLastSave="137" documentId="14_{6BA1779D-2885-C748-8AC6-FE991EB9936B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3C523115-A8F2-A14D-BD9E-BE9F8BD15A40}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17480" xr2:uid="{AFC83F48-706F-D84D-8CCC-1BE76B3461E2}"/>
+    <workbookView xWindow="19280" yWindow="500" windowWidth="30240" windowHeight="17460" xr2:uid="{AFC83F48-706F-D84D-8CCC-1BE76B3461E2}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="39">
   <si>
     <t>MM_PSF</t>
   </si>
@@ -54,81 +54,116 @@
     <t>Thermal</t>
   </si>
   <si>
+    <t>Fixed Sym Gaussian 0.01"</t>
+  </si>
+  <si>
     <t>1 keV [row#]</t>
   </si>
   <si>
-    <t># Opt 1</t>
-  </si>
-  <si>
-    <t># Opt 2</t>
-  </si>
-  <si>
-    <t># Opt 3</t>
-  </si>
-  <si>
-    <t># Opt 4</t>
-  </si>
-  <si>
-    <t># Opt 5</t>
-  </si>
-  <si>
-    <t>Total # options</t>
-  </si>
-  <si>
-    <t>Standard medialario (*)</t>
-  </si>
-  <si>
-    <t>GZ (*)</t>
-  </si>
-  <si>
-    <t>FMS tilt 0 deg (*)</t>
-  </si>
-  <si>
-    <t>0 (*)</t>
-  </si>
-  <si>
-    <t>Placement</t>
-  </si>
-  <si>
-    <t>cross</t>
-  </si>
-  <si>
-    <t>optimize</t>
-  </si>
-  <si>
-    <t>fine</t>
-  </si>
-  <si>
-    <t>-</t>
-  </si>
-  <si>
-    <t>elliptical (*)</t>
-  </si>
-  <si>
-    <t>coarse (*)</t>
-  </si>
-  <si>
-    <t>Fixed Sym Gaussian (sigma_rad=0.05 micron, sigma_azi=0.05 micron)</t>
+    <t>Standard medialario</t>
+  </si>
+  <si>
+    <t>30 deg FMS Tilt</t>
+  </si>
+  <si>
+    <t>GZ</t>
+  </si>
+  <si>
+    <t>6 keV [row#]</t>
   </si>
   <si>
     <t>Fixed Sym Gaussian 8"</t>
+  </si>
+  <si>
+    <t>Fixed Asym Gaussian 8" (ratio 7:1)</t>
+  </si>
+  <si>
+    <t>Fixed Pseudo-Voigt  8"</t>
+  </si>
+  <si>
+    <t>10% Variable Asym Gaussian 8" (ratio 7:1)</t>
+  </si>
+  <si>
+    <t>50% Variable Asym Gaussian 8" (ratio 7:1)</t>
+  </si>
+  <si>
+    <t>10% Variable Pseudo-Voigt 8" (alpha 10%)</t>
+  </si>
+  <si>
+    <t>50% Variable Pseudo-Voigt 8" (alpha 10%)</t>
+  </si>
+  <si>
+    <t>30% worse medialario</t>
+  </si>
+  <si>
+    <t>1 keV</t>
+  </si>
+  <si>
+    <t>6 keV</t>
+  </si>
+  <si>
+    <t>30% Variable Pseudo-Voigt 8" (alpha 10%)</t>
+  </si>
+  <si>
+    <t>0 deg FMS Tilt</t>
+  </si>
+  <si>
+    <t>Fixed Sym Gaussian 4.3"</t>
+  </si>
+  <si>
+    <t>Fixed Asym Gaussian 4.3" (ratio 4:1)</t>
+  </si>
+  <si>
+    <t>Fixed Pseudo-Voigt 4.3"</t>
+  </si>
+  <si>
+    <t>10% Variable Sym Gaussian 4.3"</t>
+  </si>
+  <si>
+    <t>30% Variable Sym Gaussian 4.3"</t>
+  </si>
+  <si>
+    <t>50% Variable Sym Gaussian 4.3"</t>
+  </si>
+  <si>
+    <t>10% Variable Sym Gaussian 8"</t>
+  </si>
+  <si>
+    <t>30% Variable Sym Gaussian 8"</t>
+  </si>
+  <si>
+    <t>50% Variable Sym Gaussian 8"</t>
+  </si>
+  <si>
+    <t>10% Variable Asym Gaussian 4.3" (ratio 4:1)</t>
+  </si>
+  <si>
+    <t>30% Variable Asym Gaussian 4.3" (ratio 4:1)</t>
+  </si>
+  <si>
+    <t>50% Variable Asym Gaussian 4.3" (ratio 4:1)</t>
+  </si>
+  <si>
+    <t>30% Variable Asym Gaussian 8" (ratio 7:1)</t>
+  </si>
+  <si>
+    <t>10% Variable Pseudo-Voigt 4.3" (alpha 10%)</t>
+  </si>
+  <si>
+    <t>30% Variable Pseudo-Voigt 4.3" (alpha 10%)</t>
+  </si>
+  <si>
+    <t>50% Variable Pseudo-Voigt 4.3" (alpha 10%)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FFFF0000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -145,6 +180,19 @@
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -167,10 +215,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -186,10 +235,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -509,7 +554,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC3037BA-FCD1-CB41-A0C1-80209FDB42FB}">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H26"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15.1640625" customWidth="1"/>
@@ -541,10 +586,10 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2" t="s">
         <v>5</v>
-      </c>
-      <c r="B2" t="s">
-        <v>23</v>
       </c>
       <c r="C2">
         <v>0</v>
@@ -557,12 +602,145 @@
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="B3" t="s">
+      <c r="A3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>24</v>
       </c>
     </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="B6" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="B7" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="B8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="B9" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="B10" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="B11" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="B12" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="B13" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="B14" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="B15" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="B16" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="17" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B17" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="18" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B18" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="19" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B19" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="20" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B20" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="21" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B21" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="22" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B22" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="23" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B23" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="24" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B24" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="25" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B25" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="26" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B26" t="s">
+        <v>17</v>
+      </c>
+    </row>
   </sheetData>
-  <phoneticPr fontId="2" type="noConversion"/>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -573,160 +751,97 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>1</v>
+      </c>
       <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1"/>
+      <c r="K1" s="1"/>
+      <c r="L1" s="1"/>
+      <c r="M1" s="1"/>
+      <c r="N1" s="1"/>
+      <c r="O1" s="1"/>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
         <v>6</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="B2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2">
+        <v>0</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+      <c r="E2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" t="s">
         <v>7</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E3" t="s">
         <v>8</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="N1" s="1" t="s">
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="B4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="B5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="B6" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="B7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="B8" t="s">
         <v>16</v>
       </c>
-      <c r="O1" s="1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="B2">
-        <f>COUNTIF(Sheet1!A1:A31,"&lt;&gt;")-1</f>
-        <v>1</v>
-      </c>
-      <c r="C2">
-        <f>COUNTIF(Sheet1!B1:B31,"&lt;&gt;")-1</f>
-        <v>2</v>
-      </c>
-      <c r="D2">
-        <f>COUNTIF(Sheet1!C5:C31,"&lt;&gt;")-1</f>
-        <v>-1</v>
-      </c>
-      <c r="E2">
-        <f>COUNTIF(Sheet1!D5:D31,"&lt;&gt;")-1</f>
-        <v>-1</v>
-      </c>
-      <c r="F2">
-        <f>COUNTIF(Sheet1!E5:E31,"&lt;&gt;")-1</f>
-        <v>-1</v>
-      </c>
-      <c r="K2" t="s">
-        <v>15</v>
-      </c>
-      <c r="L2" t="s">
-        <v>15</v>
-      </c>
-      <c r="M2" t="s">
-        <v>15</v>
-      </c>
-      <c r="N2" t="s">
-        <v>20</v>
-      </c>
-      <c r="O2" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="B3" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="K3" t="s">
-        <v>12</v>
-      </c>
-      <c r="L3" t="s">
-        <v>13</v>
-      </c>
-      <c r="M3" t="s">
-        <v>14</v>
-      </c>
-      <c r="N3" t="s">
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="B9" t="s">
         <v>17</v>
       </c>
-      <c r="O3" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="B4" s="2">
-        <f>B2*C2*D2*E2*F2</f>
-        <v>-2</v>
-      </c>
-      <c r="N4" t="s">
-        <v>21</v>
-      </c>
-      <c r="O4" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A10">
-        <v>2</v>
-      </c>
-      <c r="B10">
-        <v>4</v>
-      </c>
-      <c r="C10">
-        <v>2</v>
-      </c>
-      <c r="D10">
-        <v>1</v>
-      </c>
-      <c r="E10">
-        <v>1</v>
-      </c>
-      <c r="G10">
-        <f>(B10*C10*D10*E10)</f>
-        <v>8</v>
-      </c>
-      <c r="H10">
-        <f>36*G10</f>
-        <v>288</v>
-      </c>
-    </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="H11">
-        <f>25*A10*C10*D10*E10</f>
-        <v>100</v>
-      </c>
-    </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="H12">
-        <f>6*A10*B10*D10*E10</f>
-        <v>48</v>
-      </c>
-    </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="H13">
-        <f>4*A10*B10*C10*E10</f>
-        <v>64</v>
-      </c>
-    </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="H14">
-        <f>4*A10*B10*C10*D10</f>
-        <v>64</v>
-      </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="H15" s="1">
-        <f>SUM(H10:H14)</f>
-        <v>564</v>
-      </c>
+      <c r="H15" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -735,6 +850,6 @@
 
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
-  <clbl:label id="{3976fa30-1907-4356-8241-62ea5e1c0256}" enabled="1" method="Privileged" siteId="{9a5cacd0-2bef-4dd7-ac5c-7ebe1f54f495}" removed="0"/>
+  <clbl:label id="{3976fa30-1907-4356-8241-62ea5e1c0256}" enabled="1" method="Standard" siteId="{9a5cacd0-2bef-4dd7-ac5c-7ebe1f54f495}" contentBits="0" removed="0"/>
 </clbl:labelList>
 </file>
</xml_diff>